<commit_message>
Use the Assura Elevate logo and its exact gold
- Transparent logo cut from the supplied artwork, with a light-text variant for the navy bar
- Accent set to the logo gold (#E0A708), with a darker gold for small text on light surfaces
- Workbook headers and chart gold series follow the logo gold

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017kx54kpSf5ZC3j2uejwJRj
</commit_message>
<xml_diff>
--- a/samples/xlsx/AE-0001/2025-10.xlsx
+++ b/samples/xlsx/AE-0001/2025-10.xlsx
@@ -49,7 +49,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00C9971C"/>
+      <color rgb="00E0A708"/>
       <sz val="11"/>
     </font>
     <font>
@@ -106,7 +106,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C9971C"/>
+        <fgColor rgb="00E0A708"/>
       </patternFill>
     </fill>
   </fills>

</xml_diff>

<commit_message>
Monthly workbook sent from the portal, filled and locked for one client and month; uploads checked against it and reviewed before they go live
- Workbook's first sheet carries company code, name, month and a workbook reference, filled by the portal and locked
- Team emails it to the client's saved accounts address through the firm's mailbox (SMTP), or downloads a filled copy; every copy is recorded
- A returned workbook is accepted only for the client and month its reference was issued for
- Uploads are checked and summarised first, and change nothing until accepted
- Workbook colours follow the pitch deck
</commit_message>
<xml_diff>
--- a/samples/xlsx/AE-0001/2025-10.xlsx
+++ b/samples/xlsx/AE-0001/2025-10.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company &amp; Period" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company &amp; Period" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchases" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expenses" sheetId="5" state="visible" r:id="rId5"/>
@@ -48,27 +48,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00E0A708"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001F3A68"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="005A6475"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F3A68"/>
-    </font>
-    <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
@@ -76,13 +55,34 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00000000"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color rgb="00221D17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00574D3E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00DFA500"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00221D17"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -91,7 +91,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3A68"/>
+        <fgColor rgb="00221D17"/>
       </patternFill>
     </fill>
     <fill>
@@ -101,12 +101,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEF2F8"/>
+        <fgColor rgb="00F2EDDC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E0A708"/>
+        <fgColor rgb="00FAF7ED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DFA500"/>
       </patternFill>
     </fill>
   </fills>
@@ -120,7 +125,7 @@
     </border>
     <border>
       <bottom style="thin">
-        <color rgb="00D5DBE5"/>
+        <color rgb="00DDD3BC"/>
       </bottom>
     </border>
   </borders>
@@ -129,24 +134,30 @@
   </cellStyleXfs>
   <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -841,252 +852,172 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C24"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="95" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Guidance</t>
+        </is>
+      </c>
+    </row>
     <row r="2">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>ASSURA ELEVATE</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Company Code</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>AE-0001</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Client reference issued by Assura Elevate. Filled in and locked by Assura Elevate.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Monthly Data Collection Workbook</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Company Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Meridian Polymers Pvt Ltd (Demo)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Filled in and locked by Assura Elevate.</t>
         </is>
       </c>
     </row>
     <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Period (Month)</t>
+        </is>
+      </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Template version 1.0. Prepared by your in-house accountant once a month and uploaded to your Assura Elevate login.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>1. Company &amp; Period</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Fill your company code (issued by Assura Elevate), the month, and your name.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>2. One workbook a month</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Use a fresh copy each month. Uploading the same month again replaces the earlier version, and the history is kept.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>3. Paste from Tally</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Each sheet names the Tally report it comes from. Paste rows under the blue header; extra columns are ignored.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>4. Columns</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Gold headers are required. Keep the header names. Dates can be 01-09-2026, 2026-09-01 or 1-Sep-2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>5. Amounts</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Enter amounts in rupees without symbols. Negative balances (OD/CC utilisation) as minus figures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>6. Month-end positions</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Receivables, Payables, Inventory and Cash &amp; Bank are balances on the last day of the month, bill by bill.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>7. Upload</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Sign in, open Upload data, choose this file. The platform checks it and lists anything that needs fixing before it is accepted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Your role</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>You remain responsible for the books. Assura Elevate reviews, analyses and reports on the data you provide.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Sheet</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>What goes in it</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Company &amp; Period</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>One row per field. Tells the platform which company and which month this workbook covers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Every sales invoice for the month. Tally: Display &gt; Account Books &gt; Sales Register (voucher level).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Purchases</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Every purchase bill for the month (goods and services for resale or production). Tally: Purchase Register.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Expenses</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Operating expenses for the month by ledger head (salaries, rent, power, freight, finance cost and so on). One row per head is enough.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Receivables</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Every unpaid customer invoice as at month end. Tally: Display &gt; Statements of Accounts &gt; Outstandings &gt; Receivables (bill-wise).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>Payables</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Every unpaid supplier bill as at month end. Tally: Outstandings &gt; Payables (bill-wise).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Inventory</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Closing stock as at month end, item-wise. Tally: Stock Summary with Ageing Analysis, or Stock Summary plus last movement date.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Cash &amp; Bank</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Closing balance of every bank, cash, OD and CC account at month end.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>Compliance</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Status of every statutory and governance item due in or around this month.</t>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>The month this workbook is for. Filled in and locked by Assura Elevate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Workbook Reference</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>AE-0001-2025-10-SAMPLE</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Identifies this copy of the workbook, issued for this company and month only. Filled in and locked by Assura Elevate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Prepared By</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>R. Menon (Accounts)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Required. Name of the in-house accountant</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Prepared On</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>45967</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Opening Stock Value</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>15700000</v>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Needed for the first month only. Later months use the previous month's closing inventory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>69270</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Interest, rent and other non-operating income for the month</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Accountant Notes</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Anything unusual this month (one-offs, provisions, reclassifications)</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1361,150 +1292,248 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="B2:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>Field</t>
-        </is>
-      </c>
-      <c r="B1" s="6" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="C1" s="6" t="inlineStr">
-        <is>
-          <t>Guidance</t>
-        </is>
-      </c>
-    </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>Company Code</t>
-        </is>
-      </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>AE-0001</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Required. Code issued by Assura Elevate, e.g. AE-0001</t>
+          <t>ASSURA ELEVATE</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>Company Name</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>Meridian Polymers Pvt Ltd (Demo)</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Required. </t>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Monthly Data Collection Workbook</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>Period (Month)</t>
-        </is>
-      </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Required. Month the data relates to, e.g. 2026-09 or Sep-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>Prepared By</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>R. Menon (Accounts)</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Required. Name of the in-house accountant</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Prepared On</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="n">
-        <v>45967</v>
-      </c>
-      <c r="C6" s="3" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Opening Stock Value</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="n">
-        <v>15700000</v>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Needed for the first month only. Later months use the previous month's closing inventory.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Other Income</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="n">
-        <v>69270</v>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Interest, rent and other non-operating income for the month</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Accountant Notes</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Anything unusual this month (one-offs, provisions, reclassifications)</t>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Template version 1.0. Prepared by your in-house accountant once a month and uploaded to your Assura Elevate login.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>1. Company &amp; Period</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Your company, the month and the workbook reference are filled in by Assura Elevate and locked. Add your name and any notes for the month.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>2. One workbook a month</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Each month Assura Elevate sends a fresh copy made for your company and that month only. Use the copy you received for that month; another company's or another month's copy is refused.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>3. Paste from Tally</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Each sheet names the Tally report it comes from. Paste rows under the blue header; extra columns are ignored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>4. Columns</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Gold headers are required. Keep the header names. Dates can be 01-09-2026, 2026-09-01 or 1-Sep-2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>5. Amounts</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Enter amounts in rupees without symbols. Negative balances (OD/CC utilisation) as minus figures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>6. Month-end positions</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Receivables, Payables, Inventory and Cash &amp; Bank are balances on the last day of the month, bill by bill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>7. Return it</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Reply to the email with the completed workbook attached. Assura Elevate checks it is your company's copy for the month, reviews it and then adds it to your dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Your role</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>You remain responsible for the books. Assura Elevate reviews, analyses and reports on the data you provide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>What goes in it</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Company &amp; Period</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>One row per field. Tells the platform which company and which month this workbook covers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Every sales invoice for the month. Tally: Display &gt; Account Books &gt; Sales Register (voucher level).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Purchases</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Every purchase bill for the month (goods and services for resale or production). Tally: Purchase Register.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Operating expenses for the month by ledger head (salaries, rent, power, freight, finance cost and so on). One row per head is enough.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Receivables</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Every unpaid customer invoice as at month end. Tally: Display &gt; Statements of Accounts &gt; Outstandings &gt; Receivables (bill-wise).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>Payables</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Every unpaid supplier bill as at month end. Tally: Outstandings &gt; Payables (bill-wise).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Inventory</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Closing stock as at month end, item-wise. Tally: Stock Summary with Ageing Analysis, or Stock Summary plus last movement date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>Cash &amp; Bank</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Closing balance of every bank, cash, OD and CC account at month end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Status of every statutory and governance item due in or around this month.</t>
         </is>
       </c>
     </row>

</xml_diff>